<commit_message>
Per-resident analysis of the 50-cent fare, patronage, fuel price and vehicles
- Analysis notebook: four series per resident, year-on-year comparison by
  mode, correlation matrices on levels and changes, and a three-specification
  fare regression with HAC standard errors
- scripts/fetch_external_data.py: downloads and aggregates the Queensland
  fuel-price and vehicle-registration sources, with a provenance manifest
- quarterly-population-data.xlsx: ABS 3101, March 2026 release
- .gitignore: keeps the raw downloads out of the repo
- Removes analysis_population_public_transport.ipynb
</commit_message>
<xml_diff>
--- a/quarterly-population-data.xlsx
+++ b/quarterly-population-data.xlsx
@@ -17,89 +17,89 @@
     <sheet name="Enquiries" sheetId="2" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="A2060824A">Data1!$J$1:$J$10,Data1!$J$11:$J$189</definedName>
-    <definedName name="A2060824A_Data">Data1!$J$11:$J$189</definedName>
-    <definedName name="A2060824A_Latest">Data1!$J$189</definedName>
-    <definedName name="A2060825C">Data1!$B$1:$B$10,Data1!$B$11:$B$189</definedName>
-    <definedName name="A2060825C_Data">Data1!$B$11:$B$189</definedName>
-    <definedName name="A2060825C_Latest">Data1!$B$189</definedName>
-    <definedName name="A2060826F">Data1!$C$1:$C$10,Data1!$C$11:$C$189</definedName>
-    <definedName name="A2060826F_Data">Data1!$C$11:$C$189</definedName>
-    <definedName name="A2060826F_Latest">Data1!$C$189</definedName>
-    <definedName name="A2060827J">Data1!$D$1:$D$10,Data1!$D$11:$D$189</definedName>
-    <definedName name="A2060827J_Data">Data1!$D$11:$D$189</definedName>
-    <definedName name="A2060827J_Latest">Data1!$D$189</definedName>
-    <definedName name="A2060828K">Data1!$E$1:$E$10,Data1!$E$11:$E$189</definedName>
-    <definedName name="A2060828K_Data">Data1!$E$11:$E$189</definedName>
-    <definedName name="A2060828K_Latest">Data1!$E$189</definedName>
-    <definedName name="A2060829L">Data1!$F$1:$F$10,Data1!$F$11:$F$189</definedName>
-    <definedName name="A2060829L_Data">Data1!$F$11:$F$189</definedName>
-    <definedName name="A2060829L_Latest">Data1!$F$189</definedName>
-    <definedName name="A2060830W">Data1!$G$1:$G$10,Data1!$G$11:$G$189</definedName>
-    <definedName name="A2060830W_Data">Data1!$G$11:$G$189</definedName>
-    <definedName name="A2060830W_Latest">Data1!$G$189</definedName>
-    <definedName name="A2060831X">Data1!$H$1:$H$10,Data1!$H$11:$H$189</definedName>
-    <definedName name="A2060831X_Data">Data1!$H$11:$H$189</definedName>
-    <definedName name="A2060831X_Latest">Data1!$H$189</definedName>
-    <definedName name="A2060832A">Data1!$I$1:$I$10,Data1!$I$11:$I$189</definedName>
-    <definedName name="A2060832A_Data">Data1!$I$11:$I$189</definedName>
-    <definedName name="A2060832A_Latest">Data1!$I$189</definedName>
-    <definedName name="A2060833C">Data1!$S$1:$S$10,Data1!$S$11:$S$189</definedName>
-    <definedName name="A2060833C_Data">Data1!$S$11:$S$189</definedName>
-    <definedName name="A2060833C_Latest">Data1!$S$189</definedName>
-    <definedName name="A2060834F">Data1!$K$1:$K$10,Data1!$K$11:$K$189</definedName>
-    <definedName name="A2060834F_Data">Data1!$K$11:$K$189</definedName>
-    <definedName name="A2060834F_Latest">Data1!$K$189</definedName>
-    <definedName name="A2060835J">Data1!$L$1:$L$10,Data1!$L$11:$L$189</definedName>
-    <definedName name="A2060835J_Data">Data1!$L$11:$L$189</definedName>
-    <definedName name="A2060835J_Latest">Data1!$L$189</definedName>
-    <definedName name="A2060836K">Data1!$M$1:$M$10,Data1!$M$11:$M$189</definedName>
-    <definedName name="A2060836K_Data">Data1!$M$11:$M$189</definedName>
-    <definedName name="A2060836K_Latest">Data1!$M$189</definedName>
-    <definedName name="A2060837L">Data1!$N$1:$N$10,Data1!$N$11:$N$189</definedName>
-    <definedName name="A2060837L_Data">Data1!$N$11:$N$189</definedName>
-    <definedName name="A2060837L_Latest">Data1!$N$189</definedName>
-    <definedName name="A2060838R">Data1!$O$1:$O$10,Data1!$O$11:$O$189</definedName>
-    <definedName name="A2060838R_Data">Data1!$O$11:$O$189</definedName>
-    <definedName name="A2060838R_Latest">Data1!$O$189</definedName>
-    <definedName name="A2060839T">Data1!$P$1:$P$10,Data1!$P$11:$P$189</definedName>
-    <definedName name="A2060839T_Data">Data1!$P$11:$P$189</definedName>
-    <definedName name="A2060839T_Latest">Data1!$P$189</definedName>
-    <definedName name="A2060840A">Data1!$Q$1:$Q$10,Data1!$Q$11:$Q$189</definedName>
-    <definedName name="A2060840A_Data">Data1!$Q$11:$Q$189</definedName>
-    <definedName name="A2060840A_Latest">Data1!$Q$189</definedName>
-    <definedName name="A2060841C">Data1!$R$1:$R$10,Data1!$R$11:$R$189</definedName>
-    <definedName name="A2060841C_Data">Data1!$R$11:$R$189</definedName>
-    <definedName name="A2060841C_Latest">Data1!$R$189</definedName>
-    <definedName name="A2060842F">Data1!$AB$1:$AB$10,Data1!$AB$11:$AB$189</definedName>
-    <definedName name="A2060842F_Data">Data1!$AB$11:$AB$189</definedName>
-    <definedName name="A2060842F_Latest">Data1!$AB$189</definedName>
-    <definedName name="A2060843J">Data1!$T$1:$T$10,Data1!$T$11:$T$189</definedName>
-    <definedName name="A2060843J_Data">Data1!$T$11:$T$189</definedName>
-    <definedName name="A2060843J_Latest">Data1!$T$189</definedName>
-    <definedName name="A2060844K">Data1!$U$1:$U$10,Data1!$U$11:$U$189</definedName>
-    <definedName name="A2060844K_Data">Data1!$U$11:$U$189</definedName>
-    <definedName name="A2060844K_Latest">Data1!$U$189</definedName>
-    <definedName name="A2060845L">Data1!$V$1:$V$10,Data1!$V$11:$V$189</definedName>
-    <definedName name="A2060845L_Data">Data1!$V$11:$V$189</definedName>
-    <definedName name="A2060845L_Latest">Data1!$V$189</definedName>
-    <definedName name="A2060846R">Data1!$W$1:$W$10,Data1!$W$11:$W$189</definedName>
-    <definedName name="A2060846R_Data">Data1!$W$11:$W$189</definedName>
-    <definedName name="A2060846R_Latest">Data1!$W$189</definedName>
-    <definedName name="A2060847T">Data1!$X$1:$X$10,Data1!$X$11:$X$189</definedName>
-    <definedName name="A2060847T_Data">Data1!$X$11:$X$189</definedName>
-    <definedName name="A2060847T_Latest">Data1!$X$189</definedName>
-    <definedName name="A2060848V">Data1!$Y$1:$Y$10,Data1!$Y$11:$Y$189</definedName>
-    <definedName name="A2060848V_Data">Data1!$Y$11:$Y$189</definedName>
-    <definedName name="A2060848V_Latest">Data1!$Y$189</definedName>
-    <definedName name="A2060849W">Data1!$Z$1:$Z$10,Data1!$Z$11:$Z$189</definedName>
-    <definedName name="A2060849W_Data">Data1!$Z$11:$Z$189</definedName>
-    <definedName name="A2060849W_Latest">Data1!$Z$189</definedName>
-    <definedName name="A2060850F">Data1!$AA$1:$AA$10,Data1!$AA$11:$AA$189</definedName>
-    <definedName name="A2060850F_Data">Data1!$AA$11:$AA$189</definedName>
-    <definedName name="A2060850F_Latest">Data1!$AA$189</definedName>
-    <definedName name="Date_Range">Data1!$A$2:$A$10,Data1!$A$11:$A$189</definedName>
-    <definedName name="Date_Range_Data">Data1!$A$11:$A$189</definedName>
+    <definedName name="A2060824A">Data1!$J$1:$J$10,Data1!$J$11:$J$190</definedName>
+    <definedName name="A2060824A_Data">Data1!$J$11:$J$190</definedName>
+    <definedName name="A2060824A_Latest">Data1!$J$190</definedName>
+    <definedName name="A2060825C">Data1!$B$1:$B$10,Data1!$B$11:$B$190</definedName>
+    <definedName name="A2060825C_Data">Data1!$B$11:$B$190</definedName>
+    <definedName name="A2060825C_Latest">Data1!$B$190</definedName>
+    <definedName name="A2060826F">Data1!$C$1:$C$10,Data1!$C$11:$C$190</definedName>
+    <definedName name="A2060826F_Data">Data1!$C$11:$C$190</definedName>
+    <definedName name="A2060826F_Latest">Data1!$C$190</definedName>
+    <definedName name="A2060827J">Data1!$D$1:$D$10,Data1!$D$11:$D$190</definedName>
+    <definedName name="A2060827J_Data">Data1!$D$11:$D$190</definedName>
+    <definedName name="A2060827J_Latest">Data1!$D$190</definedName>
+    <definedName name="A2060828K">Data1!$E$1:$E$10,Data1!$E$11:$E$190</definedName>
+    <definedName name="A2060828K_Data">Data1!$E$11:$E$190</definedName>
+    <definedName name="A2060828K_Latest">Data1!$E$190</definedName>
+    <definedName name="A2060829L">Data1!$F$1:$F$10,Data1!$F$11:$F$190</definedName>
+    <definedName name="A2060829L_Data">Data1!$F$11:$F$190</definedName>
+    <definedName name="A2060829L_Latest">Data1!$F$190</definedName>
+    <definedName name="A2060830W">Data1!$G$1:$G$10,Data1!$G$11:$G$190</definedName>
+    <definedName name="A2060830W_Data">Data1!$G$11:$G$190</definedName>
+    <definedName name="A2060830W_Latest">Data1!$G$190</definedName>
+    <definedName name="A2060831X">Data1!$H$1:$H$10,Data1!$H$11:$H$190</definedName>
+    <definedName name="A2060831X_Data">Data1!$H$11:$H$190</definedName>
+    <definedName name="A2060831X_Latest">Data1!$H$190</definedName>
+    <definedName name="A2060832A">Data1!$I$1:$I$10,Data1!$I$11:$I$190</definedName>
+    <definedName name="A2060832A_Data">Data1!$I$11:$I$190</definedName>
+    <definedName name="A2060832A_Latest">Data1!$I$190</definedName>
+    <definedName name="A2060833C">Data1!$S$1:$S$10,Data1!$S$11:$S$190</definedName>
+    <definedName name="A2060833C_Data">Data1!$S$11:$S$190</definedName>
+    <definedName name="A2060833C_Latest">Data1!$S$190</definedName>
+    <definedName name="A2060834F">Data1!$K$1:$K$10,Data1!$K$11:$K$190</definedName>
+    <definedName name="A2060834F_Data">Data1!$K$11:$K$190</definedName>
+    <definedName name="A2060834F_Latest">Data1!$K$190</definedName>
+    <definedName name="A2060835J">Data1!$L$1:$L$10,Data1!$L$11:$L$190</definedName>
+    <definedName name="A2060835J_Data">Data1!$L$11:$L$190</definedName>
+    <definedName name="A2060835J_Latest">Data1!$L$190</definedName>
+    <definedName name="A2060836K">Data1!$M$1:$M$10,Data1!$M$11:$M$190</definedName>
+    <definedName name="A2060836K_Data">Data1!$M$11:$M$190</definedName>
+    <definedName name="A2060836K_Latest">Data1!$M$190</definedName>
+    <definedName name="A2060837L">Data1!$N$1:$N$10,Data1!$N$11:$N$190</definedName>
+    <definedName name="A2060837L_Data">Data1!$N$11:$N$190</definedName>
+    <definedName name="A2060837L_Latest">Data1!$N$190</definedName>
+    <definedName name="A2060838R">Data1!$O$1:$O$10,Data1!$O$11:$O$190</definedName>
+    <definedName name="A2060838R_Data">Data1!$O$11:$O$190</definedName>
+    <definedName name="A2060838R_Latest">Data1!$O$190</definedName>
+    <definedName name="A2060839T">Data1!$P$1:$P$10,Data1!$P$11:$P$190</definedName>
+    <definedName name="A2060839T_Data">Data1!$P$11:$P$190</definedName>
+    <definedName name="A2060839T_Latest">Data1!$P$190</definedName>
+    <definedName name="A2060840A">Data1!$Q$1:$Q$10,Data1!$Q$11:$Q$190</definedName>
+    <definedName name="A2060840A_Data">Data1!$Q$11:$Q$190</definedName>
+    <definedName name="A2060840A_Latest">Data1!$Q$190</definedName>
+    <definedName name="A2060841C">Data1!$R$1:$R$10,Data1!$R$11:$R$190</definedName>
+    <definedName name="A2060841C_Data">Data1!$R$11:$R$190</definedName>
+    <definedName name="A2060841C_Latest">Data1!$R$190</definedName>
+    <definedName name="A2060842F">Data1!$AB$1:$AB$10,Data1!$AB$11:$AB$190</definedName>
+    <definedName name="A2060842F_Data">Data1!$AB$11:$AB$190</definedName>
+    <definedName name="A2060842F_Latest">Data1!$AB$190</definedName>
+    <definedName name="A2060843J">Data1!$T$1:$T$10,Data1!$T$11:$T$190</definedName>
+    <definedName name="A2060843J_Data">Data1!$T$11:$T$190</definedName>
+    <definedName name="A2060843J_Latest">Data1!$T$190</definedName>
+    <definedName name="A2060844K">Data1!$U$1:$U$10,Data1!$U$11:$U$190</definedName>
+    <definedName name="A2060844K_Data">Data1!$U$11:$U$190</definedName>
+    <definedName name="A2060844K_Latest">Data1!$U$190</definedName>
+    <definedName name="A2060845L">Data1!$V$1:$V$10,Data1!$V$11:$V$190</definedName>
+    <definedName name="A2060845L_Data">Data1!$V$11:$V$190</definedName>
+    <definedName name="A2060845L_Latest">Data1!$V$190</definedName>
+    <definedName name="A2060846R">Data1!$W$1:$W$10,Data1!$W$11:$W$190</definedName>
+    <definedName name="A2060846R_Data">Data1!$W$11:$W$190</definedName>
+    <definedName name="A2060846R_Latest">Data1!$W$190</definedName>
+    <definedName name="A2060847T">Data1!$X$1:$X$10,Data1!$X$11:$X$190</definedName>
+    <definedName name="A2060847T_Data">Data1!$X$11:$X$190</definedName>
+    <definedName name="A2060847T_Latest">Data1!$X$190</definedName>
+    <definedName name="A2060848V">Data1!$Y$1:$Y$10,Data1!$Y$11:$Y$190</definedName>
+    <definedName name="A2060848V_Data">Data1!$Y$11:$Y$190</definedName>
+    <definedName name="A2060848V_Latest">Data1!$Y$190</definedName>
+    <definedName name="A2060849W">Data1!$Z$1:$Z$10,Data1!$Z$11:$Z$190</definedName>
+    <definedName name="A2060849W_Data">Data1!$Z$11:$Z$190</definedName>
+    <definedName name="A2060849W_Latest">Data1!$Z$190</definedName>
+    <definedName name="A2060850F">Data1!$AA$1:$AA$10,Data1!$AA$11:$AA$190</definedName>
+    <definedName name="A2060850F_Data">Data1!$AA$11:$AA$190</definedName>
+    <definedName name="A2060850F_Latest">Data1!$AA$190</definedName>
+    <definedName name="Date_Range">Data1!$A$2:$A$10,Data1!$A$11:$A$190</definedName>
+    <definedName name="Date_Range_Data">Data1!$A$11:$A$190</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -1108,10 +1108,10 @@
         <v>29738</v>
       </c>
       <c r="G12" s="9">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="H12" s="10">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I12" s="10" t="s">
         <v>36</v>
@@ -1140,10 +1140,10 @@
         <v>29738</v>
       </c>
       <c r="G13" s="9">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="H13" s="10">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I13" s="10" t="s">
         <v>36</v>
@@ -1172,10 +1172,10 @@
         <v>29738</v>
       </c>
       <c r="G14" s="9">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="H14" s="10">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I14" s="10" t="s">
         <v>36</v>
@@ -1204,10 +1204,10 @@
         <v>29738</v>
       </c>
       <c r="G15" s="9">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="H15" s="10">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I15" s="10" t="s">
         <v>36</v>
@@ -1236,10 +1236,10 @@
         <v>29738</v>
       </c>
       <c r="G16" s="9">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="H16" s="10">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I16" s="10" t="s">
         <v>36</v>
@@ -1268,10 +1268,10 @@
         <v>29738</v>
       </c>
       <c r="G17" s="9">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="H17" s="10">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I17" s="10" t="s">
         <v>36</v>
@@ -1300,10 +1300,10 @@
         <v>29738</v>
       </c>
       <c r="G18" s="9">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="H18" s="10">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I18" s="10" t="s">
         <v>36</v>
@@ -1332,10 +1332,10 @@
         <v>29738</v>
       </c>
       <c r="G19" s="9">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="H19" s="10">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I19" s="10" t="s">
         <v>36</v>
@@ -1364,10 +1364,10 @@
         <v>29738</v>
       </c>
       <c r="G20" s="9">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="H20" s="10">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I20" s="10" t="s">
         <v>36</v>
@@ -1396,10 +1396,10 @@
         <v>29738</v>
       </c>
       <c r="G21" s="9">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="H21" s="10">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I21" s="10" t="s">
         <v>36</v>
@@ -1428,10 +1428,10 @@
         <v>29738</v>
       </c>
       <c r="G22" s="9">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="H22" s="10">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I22" s="10" t="s">
         <v>36</v>
@@ -1460,10 +1460,10 @@
         <v>29738</v>
       </c>
       <c r="G23" s="9">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="H23" s="10">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I23" s="10" t="s">
         <v>36</v>
@@ -1492,10 +1492,10 @@
         <v>29738</v>
       </c>
       <c r="G24" s="9">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="H24" s="10">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I24" s="10" t="s">
         <v>36</v>
@@ -1524,10 +1524,10 @@
         <v>29738</v>
       </c>
       <c r="G25" s="9">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="H25" s="10">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I25" s="10" t="s">
         <v>36</v>
@@ -1556,10 +1556,10 @@
         <v>29738</v>
       </c>
       <c r="G26" s="9">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="H26" s="10">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I26" s="10" t="s">
         <v>36</v>
@@ -1588,10 +1588,10 @@
         <v>29738</v>
       </c>
       <c r="G27" s="9">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="H27" s="10">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I27" s="10" t="s">
         <v>36</v>
@@ -1620,10 +1620,10 @@
         <v>29738</v>
       </c>
       <c r="G28" s="9">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="H28" s="10">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I28" s="10" t="s">
         <v>36</v>
@@ -1652,10 +1652,10 @@
         <v>29738</v>
       </c>
       <c r="G29" s="9">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="H29" s="10">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I29" s="10" t="s">
         <v>36</v>
@@ -1684,10 +1684,10 @@
         <v>29738</v>
       </c>
       <c r="G30" s="9">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="H30" s="10">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I30" s="10" t="s">
         <v>36</v>
@@ -1716,10 +1716,10 @@
         <v>29738</v>
       </c>
       <c r="G31" s="9">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="H31" s="10">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I31" s="10" t="s">
         <v>36</v>
@@ -1748,10 +1748,10 @@
         <v>29738</v>
       </c>
       <c r="G32" s="9">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="H32" s="10">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I32" s="10" t="s">
         <v>36</v>
@@ -1780,10 +1780,10 @@
         <v>29738</v>
       </c>
       <c r="G33" s="9">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="H33" s="10">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I33" s="10" t="s">
         <v>36</v>
@@ -1812,10 +1812,10 @@
         <v>29738</v>
       </c>
       <c r="G34" s="9">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="H34" s="10">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I34" s="10" t="s">
         <v>36</v>
@@ -1844,10 +1844,10 @@
         <v>29738</v>
       </c>
       <c r="G35" s="9">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="H35" s="10">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I35" s="10" t="s">
         <v>36</v>
@@ -1876,10 +1876,10 @@
         <v>29738</v>
       </c>
       <c r="G36" s="9">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="H36" s="10">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I36" s="10" t="s">
         <v>36</v>
@@ -1908,10 +1908,10 @@
         <v>29738</v>
       </c>
       <c r="G37" s="9">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="H37" s="10">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I37" s="10" t="s">
         <v>36</v>
@@ -1940,10 +1940,10 @@
         <v>29738</v>
       </c>
       <c r="G38" s="9">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="H38" s="10">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I38" s="10" t="s">
         <v>36</v>
@@ -2005,7 +2005,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AB189"/>
+  <dimension ref="A1:AB190"/>
   <sheetFormatPr defaultColWidth="14.7109375" defaultRowHeight="11.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="16384" width="14.7109375" style="1"/>
@@ -2615,85 +2615,85 @@
         <v>33</v>
       </c>
       <c r="B8" s="6">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="C8" s="6">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="D8" s="6">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="E8" s="6">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="F8" s="6">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="G8" s="6">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="H8" s="6">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="I8" s="6">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="J8" s="6">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="K8" s="6">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="L8" s="6">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="M8" s="6">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="N8" s="6">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="O8" s="6">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="P8" s="6">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="Q8" s="6">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="R8" s="6">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="S8" s="6">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="T8" s="6">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="U8" s="6">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="V8" s="6">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="W8" s="6">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="X8" s="6">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="Y8" s="6">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="Z8" s="6">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="AA8" s="6">
-        <v>45992</v>
+        <v>46082</v>
       </c>
       <c r="AB8" s="6">
-        <v>45992</v>
+        <v>46082</v>
       </c>
     </row>
     <row r="9" spans="1:28" x14ac:dyDescent="0.2">
@@ -2701,85 +2701,85 @@
         <v>34</v>
       </c>
       <c r="B9" s="1">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C9" s="1">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D9" s="1">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="E9" s="1">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F9" s="1">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="G9" s="1">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="H9" s="1">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I9" s="1">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="J9" s="1">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="K9" s="1">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="L9" s="1">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="M9" s="1">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="N9" s="1">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="O9" s="1">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="P9" s="1">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="Q9" s="1">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="R9" s="1">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="S9" s="1">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="T9" s="1">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="U9" s="1">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="V9" s="1">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="W9" s="1">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="X9" s="1">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="Y9" s="1">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="Z9" s="1">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="AA9" s="1">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="AB9" s="1">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="10" spans="1:28" x14ac:dyDescent="0.2">
@@ -17751,85 +17751,85 @@
         <v>45536</v>
       </c>
       <c r="B184" s="8">
-        <v>4239404</v>
+        <v>4239562</v>
       </c>
       <c r="C184" s="8">
-        <v>3446646</v>
+        <v>3445298</v>
       </c>
       <c r="D184" s="8">
-        <v>2771119</v>
+        <v>2771391</v>
       </c>
       <c r="E184" s="8">
-        <v>933367</v>
+        <v>933517</v>
       </c>
       <c r="F184" s="8">
-        <v>1506972</v>
+        <v>1506643</v>
       </c>
       <c r="G184" s="8">
-        <v>285350</v>
+        <v>285324</v>
       </c>
       <c r="H184" s="8">
-        <v>134723</v>
+        <v>134748</v>
       </c>
       <c r="I184" s="8">
-        <v>235901</v>
+        <v>235909</v>
       </c>
       <c r="J184" s="8">
-        <v>13556115</v>
+        <v>13555027</v>
       </c>
       <c r="K184" s="8">
-        <v>4279493</v>
+        <v>4279944</v>
       </c>
       <c r="L184" s="8">
-        <v>3535059</v>
+        <v>3533709</v>
       </c>
       <c r="M184" s="8">
-        <v>2824284</v>
+        <v>2824175</v>
       </c>
       <c r="N184" s="8">
-        <v>953451</v>
+        <v>953593</v>
       </c>
       <c r="O184" s="8">
-        <v>1489171</v>
+        <v>1488910</v>
       </c>
       <c r="P184" s="8">
-        <v>289989</v>
+        <v>290048</v>
       </c>
       <c r="Q184" s="8">
-        <v>127283</v>
+        <v>127278</v>
       </c>
       <c r="R184" s="8">
-        <v>243951</v>
+        <v>243964</v>
       </c>
       <c r="S184" s="8">
-        <v>13745034</v>
+        <v>13743978</v>
       </c>
       <c r="T184" s="8">
-        <v>8518897</v>
+        <v>8519506</v>
       </c>
       <c r="U184" s="8">
-        <v>6981705</v>
+        <v>6979007</v>
       </c>
       <c r="V184" s="8">
-        <v>5595403</v>
+        <v>5595566</v>
       </c>
       <c r="W184" s="8">
-        <v>1886818</v>
+        <v>1887110</v>
       </c>
       <c r="X184" s="8">
-        <v>2996143</v>
+        <v>2995553</v>
       </c>
       <c r="Y184" s="8">
-        <v>575339</v>
+        <v>575372</v>
       </c>
       <c r="Z184" s="8">
-        <v>262006</v>
+        <v>262026</v>
       </c>
       <c r="AA184" s="8">
-        <v>479852</v>
+        <v>479873</v>
       </c>
       <c r="AB184" s="8">
-        <v>27301149</v>
+        <v>27299005</v>
       </c>
     </row>
     <row r="185" spans="1:28" x14ac:dyDescent="0.2">
@@ -17837,85 +17837,85 @@
         <v>45627</v>
       </c>
       <c r="B185" s="8">
-        <v>4247126</v>
+        <v>4248239</v>
       </c>
       <c r="C185" s="8">
-        <v>3456807</v>
+        <v>3456257</v>
       </c>
       <c r="D185" s="8">
-        <v>2782878</v>
+        <v>2783307</v>
       </c>
       <c r="E185" s="8">
-        <v>935156</v>
+        <v>935368</v>
       </c>
       <c r="F185" s="8">
-        <v>1514477</v>
+        <v>1514455</v>
       </c>
       <c r="G185" s="8">
-        <v>285850</v>
+        <v>285834</v>
       </c>
       <c r="H185" s="8">
-        <v>135481</v>
+        <v>135531</v>
       </c>
       <c r="I185" s="8">
-        <v>236284</v>
+        <v>236367</v>
       </c>
       <c r="J185" s="8">
-        <v>13596696</v>
+        <v>13597992</v>
       </c>
       <c r="K185" s="8">
-        <v>4289348</v>
+        <v>4290438</v>
       </c>
       <c r="L185" s="8">
-        <v>3547791</v>
+        <v>3547553</v>
       </c>
       <c r="M185" s="8">
-        <v>2837084</v>
+        <v>2837092</v>
       </c>
       <c r="N185" s="8">
-        <v>955669</v>
+        <v>955856</v>
       </c>
       <c r="O185" s="8">
-        <v>1496586</v>
+        <v>1496742</v>
       </c>
       <c r="P185" s="8">
-        <v>290352</v>
+        <v>290437</v>
       </c>
       <c r="Q185" s="8">
-        <v>127757</v>
+        <v>127752</v>
       </c>
       <c r="R185" s="8">
-        <v>244885</v>
+        <v>244891</v>
       </c>
       <c r="S185" s="8">
-        <v>13791833</v>
+        <v>13793133</v>
       </c>
       <c r="T185" s="8">
-        <v>8536474</v>
+        <v>8538677</v>
       </c>
       <c r="U185" s="8">
-        <v>7004598</v>
+        <v>7003810</v>
       </c>
       <c r="V185" s="8">
-        <v>5619962</v>
+        <v>5620399</v>
       </c>
       <c r="W185" s="8">
-        <v>1890825</v>
+        <v>1891224</v>
       </c>
       <c r="X185" s="8">
-        <v>3011063</v>
+        <v>3011197</v>
       </c>
       <c r="Y185" s="8">
-        <v>576202</v>
+        <v>576271</v>
       </c>
       <c r="Z185" s="8">
-        <v>263238</v>
+        <v>263283</v>
       </c>
       <c r="AA185" s="8">
-        <v>481169</v>
+        <v>481258</v>
       </c>
       <c r="AB185" s="8">
-        <v>27388529</v>
+        <v>27391125</v>
       </c>
     </row>
     <row r="186" spans="1:28" x14ac:dyDescent="0.2">
@@ -17923,85 +17923,85 @@
         <v>45717</v>
       </c>
       <c r="B186" s="8">
-        <v>4265029</v>
+        <v>4265007</v>
       </c>
       <c r="C186" s="8">
-        <v>3477144</v>
+        <v>3475582</v>
       </c>
       <c r="D186" s="8">
-        <v>2797145</v>
+        <v>2797919</v>
       </c>
       <c r="E186" s="8">
-        <v>938722</v>
+        <v>938886</v>
       </c>
       <c r="F186" s="8">
-        <v>1525681</v>
+        <v>1525289</v>
       </c>
       <c r="G186" s="8">
-        <v>286332</v>
+        <v>286335</v>
       </c>
       <c r="H186" s="8">
-        <v>136440</v>
+        <v>136518</v>
       </c>
       <c r="I186" s="8">
-        <v>237101</v>
+        <v>237241</v>
       </c>
       <c r="J186" s="8">
-        <v>13666234</v>
+        <v>13665408</v>
       </c>
       <c r="K186" s="8">
-        <v>4307569</v>
+        <v>4308127</v>
       </c>
       <c r="L186" s="8">
-        <v>3570087</v>
+        <v>3569148</v>
       </c>
       <c r="M186" s="8">
-        <v>2851540</v>
+        <v>2851464</v>
       </c>
       <c r="N186" s="8">
-        <v>959487</v>
+        <v>959563</v>
       </c>
       <c r="O186" s="8">
-        <v>1506980</v>
+        <v>1506735</v>
       </c>
       <c r="P186" s="8">
-        <v>290870</v>
+        <v>290962</v>
       </c>
       <c r="Q186" s="8">
-        <v>128459</v>
+        <v>128416</v>
       </c>
       <c r="R186" s="8">
-        <v>246183</v>
+        <v>246221</v>
       </c>
       <c r="S186" s="8">
-        <v>13863541</v>
+        <v>13863014</v>
       </c>
       <c r="T186" s="8">
-        <v>8572598</v>
+        <v>8573134</v>
       </c>
       <c r="U186" s="8">
-        <v>7047231</v>
+        <v>7044730</v>
       </c>
       <c r="V186" s="8">
-        <v>5648685</v>
+        <v>5649383</v>
       </c>
       <c r="W186" s="8">
-        <v>1898209</v>
+        <v>1898449</v>
       </c>
       <c r="X186" s="8">
-        <v>3032661</v>
+        <v>3032024</v>
       </c>
       <c r="Y186" s="8">
-        <v>577202</v>
+        <v>577297</v>
       </c>
       <c r="Z186" s="8">
-        <v>264899</v>
+        <v>264934</v>
       </c>
       <c r="AA186" s="8">
-        <v>483284</v>
+        <v>483462</v>
       </c>
       <c r="AB186" s="8">
-        <v>27529775</v>
+        <v>27528422</v>
       </c>
     </row>
     <row r="187" spans="1:28" x14ac:dyDescent="0.2">
@@ -18009,85 +18009,85 @@
         <v>45809</v>
       </c>
       <c r="B187" s="8">
-        <v>4273829</v>
+        <v>4272236</v>
       </c>
       <c r="C187" s="8">
-        <v>3487921</v>
+        <v>3484720</v>
       </c>
       <c r="D187" s="8">
-        <v>2807860</v>
+        <v>2808312</v>
       </c>
       <c r="E187" s="8">
-        <v>940224</v>
+        <v>940273</v>
       </c>
       <c r="F187" s="8">
-        <v>1532726</v>
+        <v>1532010</v>
       </c>
       <c r="G187" s="8">
-        <v>286619</v>
+        <v>286569</v>
       </c>
       <c r="H187" s="8">
-        <v>137067</v>
+        <v>137151</v>
       </c>
       <c r="I187" s="8">
-        <v>237727</v>
+        <v>237819</v>
       </c>
       <c r="J187" s="8">
-        <v>13706621</v>
+        <v>13701729</v>
       </c>
       <c r="K187" s="8">
-        <v>4316284</v>
+        <v>4315133</v>
       </c>
       <c r="L187" s="8">
-        <v>3581935</v>
+        <v>3579321</v>
       </c>
       <c r="M187" s="8">
-        <v>2862055</v>
+        <v>2861891</v>
       </c>
       <c r="N187" s="8">
-        <v>961391</v>
+        <v>961379</v>
       </c>
       <c r="O187" s="8">
-        <v>1513483</v>
+        <v>1512956</v>
       </c>
       <c r="P187" s="8">
-        <v>291151</v>
+        <v>291258</v>
       </c>
       <c r="Q187" s="8">
-        <v>128828</v>
+        <v>128827</v>
       </c>
       <c r="R187" s="8">
-        <v>246908</v>
+        <v>246862</v>
       </c>
       <c r="S187" s="8">
-        <v>13904405</v>
+        <v>13900010</v>
       </c>
       <c r="T187" s="8">
-        <v>8590113</v>
+        <v>8587369</v>
       </c>
       <c r="U187" s="8">
-        <v>7069856</v>
+        <v>7064041</v>
       </c>
       <c r="V187" s="8">
-        <v>5669915</v>
+        <v>5670203</v>
       </c>
       <c r="W187" s="8">
-        <v>1901615</v>
+        <v>1901652</v>
       </c>
       <c r="X187" s="8">
-        <v>3046209</v>
+        <v>3044966</v>
       </c>
       <c r="Y187" s="8">
-        <v>577770</v>
+        <v>577827</v>
       </c>
       <c r="Z187" s="8">
-        <v>265895</v>
+        <v>265978</v>
       </c>
       <c r="AA187" s="8">
-        <v>484635</v>
+        <v>484681</v>
       </c>
       <c r="AB187" s="8">
-        <v>27611026</v>
+        <v>27601739</v>
       </c>
     </row>
     <row r="188" spans="1:28" x14ac:dyDescent="0.2">
@@ -18095,85 +18095,85 @@
         <v>45901</v>
       </c>
       <c r="B188" s="8">
-        <v>4290291</v>
+        <v>4287798</v>
       </c>
       <c r="C188" s="8">
-        <v>3502600</v>
+        <v>3499160</v>
       </c>
       <c r="D188" s="8">
-        <v>2819330</v>
+        <v>2819896</v>
       </c>
       <c r="E188" s="8">
-        <v>943119</v>
+        <v>943250</v>
       </c>
       <c r="F188" s="8">
-        <v>1542045</v>
+        <v>1541465</v>
       </c>
       <c r="G188" s="8">
-        <v>286814</v>
+        <v>286795</v>
       </c>
       <c r="H188" s="8">
-        <v>137725</v>
+        <v>137812</v>
       </c>
       <c r="I188" s="8">
-        <v>238377</v>
+        <v>238484</v>
       </c>
       <c r="J188" s="8">
-        <v>13762955</v>
+        <v>13757303</v>
       </c>
       <c r="K188" s="8">
-        <v>4332210</v>
+        <v>4330334</v>
       </c>
       <c r="L188" s="8">
-        <v>3597261</v>
+        <v>3594716</v>
       </c>
       <c r="M188" s="8">
-        <v>2873330</v>
+        <v>2873350</v>
       </c>
       <c r="N188" s="8">
-        <v>963951</v>
+        <v>964019</v>
       </c>
       <c r="O188" s="8">
-        <v>1521776</v>
+        <v>1521373</v>
       </c>
       <c r="P188" s="8">
-        <v>291512</v>
+        <v>291644</v>
       </c>
       <c r="Q188" s="8">
-        <v>129242</v>
+        <v>129276</v>
       </c>
       <c r="R188" s="8">
-        <v>247781</v>
+        <v>247713</v>
       </c>
       <c r="S188" s="8">
-        <v>13959430</v>
+        <v>13954803</v>
       </c>
       <c r="T188" s="8">
-        <v>8622501</v>
+        <v>8618132</v>
       </c>
       <c r="U188" s="8">
-        <v>7099861</v>
+        <v>7093876</v>
       </c>
       <c r="V188" s="8">
-        <v>5692660</v>
+        <v>5693246</v>
       </c>
       <c r="W188" s="8">
-        <v>1907070</v>
+        <v>1907269</v>
       </c>
       <c r="X188" s="8">
-        <v>3063821</v>
+        <v>3062838</v>
       </c>
       <c r="Y188" s="8">
-        <v>578326</v>
+        <v>578439</v>
       </c>
       <c r="Z188" s="8">
-        <v>266967</v>
+        <v>267088</v>
       </c>
       <c r="AA188" s="8">
-        <v>486158</v>
+        <v>486197</v>
       </c>
       <c r="AB188" s="8">
-        <v>27722385</v>
+        <v>27712106</v>
       </c>
     </row>
     <row r="189" spans="1:28" x14ac:dyDescent="0.2">
@@ -18181,85 +18181,171 @@
         <v>45992</v>
       </c>
       <c r="B189" s="8">
-        <v>4298725</v>
+        <v>4295355</v>
       </c>
       <c r="C189" s="8">
-        <v>3513133</v>
+        <v>3509636</v>
       </c>
       <c r="D189" s="8">
-        <v>2828745</v>
+        <v>2829532</v>
       </c>
       <c r="E189" s="8">
-        <v>944711</v>
+        <v>944825</v>
       </c>
       <c r="F189" s="8">
-        <v>1548422</v>
+        <v>1547937</v>
       </c>
       <c r="G189" s="8">
-        <v>287189</v>
+        <v>287103</v>
       </c>
       <c r="H189" s="8">
-        <v>138051</v>
+        <v>138167</v>
       </c>
       <c r="I189" s="8">
-        <v>238717</v>
+        <v>238817</v>
       </c>
       <c r="J189" s="8">
-        <v>13800350</v>
+        <v>13794018</v>
       </c>
       <c r="K189" s="8">
-        <v>4342360</v>
+        <v>4339845</v>
       </c>
       <c r="L189" s="8">
-        <v>3608780</v>
+        <v>3606380</v>
       </c>
       <c r="M189" s="8">
-        <v>2883379</v>
+        <v>2883794</v>
       </c>
       <c r="N189" s="8">
-        <v>965842</v>
+        <v>965955</v>
       </c>
       <c r="O189" s="8">
-        <v>1528106</v>
+        <v>1527927</v>
       </c>
       <c r="P189" s="8">
-        <v>291921</v>
+        <v>291982</v>
       </c>
       <c r="Q189" s="8">
-        <v>129427</v>
+        <v>129536</v>
       </c>
       <c r="R189" s="8">
-        <v>248485</v>
+        <v>248442</v>
       </c>
       <c r="S189" s="8">
-        <v>14000673</v>
+        <v>13996245</v>
       </c>
       <c r="T189" s="8">
-        <v>8641085</v>
+        <v>8635200</v>
       </c>
       <c r="U189" s="8">
-        <v>7121913</v>
+        <v>7116016</v>
       </c>
       <c r="V189" s="8">
-        <v>5712124</v>
+        <v>5713326</v>
       </c>
       <c r="W189" s="8">
-        <v>1910553</v>
+        <v>1910780</v>
       </c>
       <c r="X189" s="8">
-        <v>3076528</v>
+        <v>3075864</v>
       </c>
       <c r="Y189" s="8">
-        <v>579110</v>
+        <v>579085</v>
       </c>
       <c r="Z189" s="8">
-        <v>267478</v>
+        <v>267703</v>
       </c>
       <c r="AA189" s="8">
-        <v>487202</v>
+        <v>487259</v>
       </c>
       <c r="AB189" s="8">
-        <v>27801023</v>
+        <v>27790263</v>
+      </c>
+    </row>
+    <row r="190" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A190" s="9">
+        <v>46082</v>
+      </c>
+      <c r="B190" s="8">
+        <v>4312364</v>
+      </c>
+      <c r="C190" s="8">
+        <v>3527662</v>
+      </c>
+      <c r="D190" s="8">
+        <v>2842768</v>
+      </c>
+      <c r="E190" s="8">
+        <v>947965</v>
+      </c>
+      <c r="F190" s="8">
+        <v>1559010</v>
+      </c>
+      <c r="G190" s="8">
+        <v>287996</v>
+      </c>
+      <c r="H190" s="8">
+        <v>138877</v>
+      </c>
+      <c r="I190" s="8">
+        <v>239880</v>
+      </c>
+      <c r="J190" s="8">
+        <v>13859185</v>
+      </c>
+      <c r="K190" s="8">
+        <v>4357741</v>
+      </c>
+      <c r="L190" s="8">
+        <v>3626559</v>
+      </c>
+      <c r="M190" s="8">
+        <v>2896693</v>
+      </c>
+      <c r="N190" s="8">
+        <v>968871</v>
+      </c>
+      <c r="O190" s="8">
+        <v>1537212</v>
+      </c>
+      <c r="P190" s="8">
+        <v>292695</v>
+      </c>
+      <c r="Q190" s="8">
+        <v>130022</v>
+      </c>
+      <c r="R190" s="8">
+        <v>249788</v>
+      </c>
+      <c r="S190" s="8">
+        <v>14061965</v>
+      </c>
+      <c r="T190" s="8">
+        <v>8670105</v>
+      </c>
+      <c r="U190" s="8">
+        <v>7154221</v>
+      </c>
+      <c r="V190" s="8">
+        <v>5739461</v>
+      </c>
+      <c r="W190" s="8">
+        <v>1916836</v>
+      </c>
+      <c r="X190" s="8">
+        <v>3096222</v>
+      </c>
+      <c r="Y190" s="8">
+        <v>580691</v>
+      </c>
+      <c r="Z190" s="8">
+        <v>268899</v>
+      </c>
+      <c r="AA190" s="8">
+        <v>489668</v>
+      </c>
+      <c r="AB190" s="8">
+        <v>27921150</v>
       </c>
     </row>
   </sheetData>

</xml_diff>